<commit_message>
add: update W4 Sparklines, Advanced Charting, and Trendlines Excel files; add C2-W4 Assessment and Practice Challenge files
</commit_message>
<xml_diff>
--- a/02-intermediate-1/material_curso/modulo-04/challenge/_828fea7066b7eae714d4342077263cbc_C2-W4-Practice-Challenge-Solution.xlsx
+++ b/02-intermediate-1/material_curso/modulo-04/challenge/_828fea7066b7eae714d4342077263cbc_C2-W4-Practice-Challenge-Solution.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="18201"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mq20084022\Google Drive\Excel MOOC\002 Course 2 - Intermediate I\04 Week 4\04 Assessment\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jorge\Proyectos\ExcelLearning\02-intermediate-1\material_curso\modulo-04\challenge\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2399DAA-CBCE-497F-9B38-90AEBB7AAD33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20736" windowHeight="11760" tabRatio="537"/>
+    <workbookView xWindow="4965" yWindow="4965" windowWidth="14430" windowHeight="7755" tabRatio="537" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions " sheetId="14" r:id="rId1"/>
@@ -37,10 +38,22 @@
     <definedName name="Student_number">'Students-database'!$C$8:$C$255</definedName>
     <definedName name="Total_Payment">'Students-database'!$R$8:$R$255</definedName>
   </definedNames>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -3349,11 +3362,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3766,7 +3779,7 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -3775,7 +3788,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3790,7 +3803,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3815,7 +3828,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3840,7 +3853,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -3863,7 +3876,7 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3917,36 +3930,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -3954,7 +3937,19 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -3980,15 +3975,34 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
-    <cellStyle name="MQ Body" xfId="6"/>
-    <cellStyle name="MQ Heading 1" xfId="4"/>
+    <cellStyle name="MQ Body" xfId="6" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="MQ Heading 1" xfId="4" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2 2" xfId="2"/>
-    <cellStyle name="Normal 4" xfId="3"/>
-    <cellStyle name="Title 2" xfId="5"/>
+    <cellStyle name="Normal 2 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Normal 4" xfId="3" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Title 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
   <dxfs count="5">
     <dxf>
@@ -4095,7 +4109,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -4194,7 +4208,7 @@
                     <a:cs typeface="+mn-cs"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:endParaRPr lang="en-US"/>
+                <a:endParaRPr lang="es-419"/>
               </a:p>
             </c:txPr>
             <c:showLegendKey val="0"/>
@@ -4309,7 +4323,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -4339,7 +4353,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-US"/>
+      <a:endParaRPr lang="es-419"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4401,7 +4415,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -4560,7 +4574,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -4590,7 +4604,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-US"/>
+      <a:endParaRPr lang="es-419"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4652,7 +4666,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -4708,7 +4722,7 @@
             <c:numRef>
               <c:f>Dashboard!$B$26:$B$28</c:f>
               <c:numCache>
-                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:formatCode>_-"$"* #,##0.00_-;\-"$"* #,##0.00_-;_-"$"* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>2008800</c:v>
@@ -4773,7 +4787,7 @@
             <c:numRef>
               <c:f>Dashboard!$C$26:$C$28</c:f>
               <c:numCache>
-                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:formatCode>_-"$"* #,##0.00_-;\-"$"* #,##0.00_-;_-"$"* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>572400</c:v>
@@ -4838,7 +4852,7 @@
             <c:numRef>
               <c:f>Dashboard!$D$26:$D$28</c:f>
               <c:numCache>
-                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:formatCode>_-"$"* #,##0.00_-;\-"$"* #,##0.00_-;_-"$"* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>963900</c:v>
@@ -4903,7 +4917,7 @@
             <c:numRef>
               <c:f>Dashboard!$E$26:$E$28</c:f>
               <c:numCache>
-                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:formatCode>_-"$"* #,##0.00_-;\-"$"* #,##0.00_-;_-"$"* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>472500</c:v>
@@ -4977,7 +4991,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="es-419"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="661879712"/>
@@ -5008,7 +5022,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:numFmt formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -5036,7 +5050,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="es-419"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="654721488"/>
@@ -5078,7 +5092,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -5108,7 +5122,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-US"/>
+      <a:endParaRPr lang="es-419"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -5170,7 +5184,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -5438,7 +5452,7 @@
             <c:numRef>
               <c:f>Dashboard!$E$34:$E$36</c:f>
               <c:numCache>
-                <c:formatCode>_("$"* #,##0.00_);_("$"* \(#,##0.00\);_("$"* "-"??_);_(@_)</c:formatCode>
+                <c:formatCode>_-"$"* #,##0.00_-;\-"$"* #,##0.00_-;_-"$"* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>2033100</c:v>
@@ -5513,7 +5527,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="es-419"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="669463056"/>
@@ -5572,7 +5586,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="es-419"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="440221920"/>
@@ -5586,7 +5600,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="r"/>
-        <c:numFmt formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)" sourceLinked="1"/>
+        <c:numFmt formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -5614,7 +5628,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="es-419"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="555638064"/>
@@ -5674,7 +5688,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -5704,7 +5718,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-US"/>
+      <a:endParaRPr lang="es-419"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -5755,7 +5769,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="es-419"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -5837,10 +5851,24 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
+                  <a:endParaRPr lang="es-419"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
           </c:trendline>
           <c:val>
             <c:numRef>
@@ -5919,7 +5947,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="es-419"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="533399872"/>
@@ -5978,7 +6006,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="es-419"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="671841408"/>
@@ -6019,7 +6047,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-US"/>
+      <a:endParaRPr lang="es-419"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -10745,21 +10773,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P54"/>
-  <sheetFormatPr defaultColWidth="9.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="8" width="9.88671875" style="36"/>
-    <col min="9" max="12" width="12.33203125" style="36" customWidth="1"/>
-    <col min="13" max="13" width="39.5546875" style="36" customWidth="1"/>
-    <col min="14" max="16" width="12.33203125" style="36" customWidth="1"/>
-    <col min="17" max="16384" width="9.88671875" style="36"/>
+    <col min="1" max="8" width="9.85546875" style="36"/>
+    <col min="9" max="12" width="12.28515625" style="36" customWidth="1"/>
+    <col min="13" max="13" width="39.5703125" style="36" customWidth="1"/>
+    <col min="14" max="16" width="12.28515625" style="36" customWidth="1"/>
+    <col min="17" max="16384" width="9.85546875" style="36"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16">
       <c r="H1" s="41"/>
     </row>
-    <row r="2" spans="1:16" ht="34.799999999999997" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:16" ht="34.5">
       <c r="H2" s="48" t="s">
         <v>292</v>
       </c>
@@ -10772,10 +10800,10 @@
       <c r="O2" s="49"/>
       <c r="P2" s="49"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16">
       <c r="H3" s="41"/>
     </row>
-    <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:16" ht="30">
       <c r="H4" s="50" t="s">
         <v>293</v>
       </c>
@@ -10788,10 +10816,10 @@
       <c r="O4" s="51"/>
       <c r="P4" s="51"/>
     </row>
-    <row r="5" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="15.75" thickBot="1">
       <c r="H5" s="41"/>
     </row>
-    <row r="6" spans="1:16" ht="31.8" thickBot="1" x14ac:dyDescent="0.65">
+    <row r="6" spans="1:16" ht="32.25" thickBot="1">
       <c r="H6" s="41"/>
       <c r="I6" s="52" t="s">
         <v>291</v>
@@ -10804,10 +10832,10 @@
       <c r="O6" s="54"/>
       <c r="P6" s="39"/>
     </row>
-    <row r="7" spans="1:16" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:16" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:16" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" customFormat="1"/>
+    <row r="8" spans="1:16" customFormat="1"/>
+    <row r="9" spans="1:16" customFormat="1"/>
+    <row r="10" spans="1:16" ht="18.75" thickBot="1">
       <c r="A10" s="40" t="s">
         <v>294</v>
       </c>
@@ -10827,7 +10855,7 @@
       <c r="O10"/>
       <c r="P10"/>
     </row>
-    <row r="11" spans="1:16" ht="12.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="12.6" customHeight="1" thickTop="1">
       <c r="A11" s="38"/>
       <c r="B11" s="38"/>
       <c r="C11" s="38"/>
@@ -10845,7 +10873,7 @@
       <c r="O11"/>
       <c r="P11"/>
     </row>
-    <row r="12" spans="1:16" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="49.9" customHeight="1">
       <c r="A12" s="55" t="s">
         <v>558</v>
       </c>
@@ -10864,9 +10892,9 @@
       <c r="N12" s="55"/>
       <c r="O12" s="55"/>
     </row>
-    <row r="13" spans="1:16" customFormat="1" ht="9" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:16" customFormat="1" ht="5.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:16" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" customFormat="1" ht="9" customHeight="1"/>
+    <row r="14" spans="1:16" customFormat="1" ht="5.45" customHeight="1"/>
+    <row r="15" spans="1:16" ht="18.75" thickBot="1">
       <c r="A15" s="40" t="s">
         <v>290</v>
       </c>
@@ -10880,7 +10908,7 @@
       <c r="I15" s="37"/>
       <c r="M15" s="23"/>
     </row>
-    <row r="16" spans="1:16" ht="10.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="10.5" customHeight="1" thickTop="1">
       <c r="A16" s="38"/>
       <c r="B16" s="38"/>
       <c r="C16" s="38"/>
@@ -10891,30 +10919,30 @@
       <c r="H16" s="38"/>
       <c r="I16" s="37"/>
     </row>
-    <row r="17" spans="1:2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" customFormat="1">
       <c r="A17" t="s">
         <v>559</v>
       </c>
     </row>
-    <row r="18" spans="1:2" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="1:2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" customFormat="1"/>
+    <row r="19" spans="1:2" customFormat="1">
       <c r="A19" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="20" spans="1:2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" customFormat="1">
       <c r="A20" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="21" spans="1:2" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" customFormat="1"/>
+    <row r="22" spans="1:2" customFormat="1">
       <c r="A22" t="s">
         <v>564</v>
       </c>
     </row>
-    <row r="23" spans="1:2" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="1:2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" customFormat="1"/>
+    <row r="24" spans="1:2" customFormat="1">
       <c r="A24" s="36">
         <v>1</v>
       </c>
@@ -10922,7 +10950,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2">
       <c r="A25" s="36">
         <v>2</v>
       </c>
@@ -10930,7 +10958,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2">
       <c r="A26" s="36">
         <v>3</v>
       </c>
@@ -10938,7 +10966,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2">
       <c r="A27" s="36">
         <v>4</v>
       </c>
@@ -10946,7 +10974,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2">
       <c r="A28" s="36">
         <v>5</v>
       </c>
@@ -10954,7 +10982,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2">
       <c r="A29" s="36">
         <v>6</v>
       </c>
@@ -10962,7 +10990,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2">
       <c r="A30" s="36">
         <v>7</v>
       </c>
@@ -10970,7 +10998,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2">
       <c r="A31" s="36">
         <v>8</v>
       </c>
@@ -10978,7 +11006,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2">
       <c r="A32" s="36">
         <v>9</v>
       </c>
@@ -10986,7 +11014,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2">
       <c r="A33" s="36">
         <v>10</v>
       </c>
@@ -10994,7 +11022,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2">
       <c r="A34" s="36">
         <v>11</v>
       </c>
@@ -11002,7 +11030,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2">
       <c r="A35" s="36">
         <v>12</v>
       </c>
@@ -11010,7 +11038,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2">
       <c r="A36" s="36">
         <v>13</v>
       </c>
@@ -11018,7 +11046,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2">
       <c r="A37" s="36">
         <v>14</v>
       </c>
@@ -11026,7 +11054,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2">
       <c r="A38" s="36">
         <v>15</v>
       </c>
@@ -11034,7 +11062,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2">
       <c r="A39" s="36">
         <v>16</v>
       </c>
@@ -11042,7 +11070,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2">
       <c r="A40" s="36">
         <v>17</v>
       </c>
@@ -11050,7 +11078,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2">
       <c r="A41" s="36">
         <v>18</v>
       </c>
@@ -11058,7 +11086,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2">
       <c r="A42" s="36">
         <v>19</v>
       </c>
@@ -11066,32 +11094,32 @@
         <v>554</v>
       </c>
     </row>
-    <row r="43" spans="1:2" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="44" spans="1:2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" customFormat="1"/>
+    <row r="44" spans="1:2" customFormat="1">
       <c r="A44" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="45" spans="1:2" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" customFormat="1"/>
+    <row r="48" spans="1:2">
       <c r="A48" s="19"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1">
       <c r="A49" s="42"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1">
       <c r="A50" s="42"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1">
       <c r="A51" s="19"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1">
       <c r="A52" s="19"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1">
       <c r="A53" s="19"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:1">
       <c r="A54" s="19"/>
     </row>
   </sheetData>
@@ -11109,25 +11137,25 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="C1:R255"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="C1:R257"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.5546875" customWidth="1"/>
-    <col min="2" max="2" width="2.109375" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" customWidth="1"/>
-    <col min="7" max="7" width="13.88671875" customWidth="1"/>
-    <col min="8" max="8" width="12.109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" style="1" customWidth="1"/>
-    <col min="10" max="14" width="11.33203125" style="1" customWidth="1"/>
-    <col min="15" max="17" width="11.33203125" customWidth="1"/>
-    <col min="18" max="18" width="13.109375" customWidth="1"/>
+    <col min="1" max="1" width="2.5703125" customWidth="1"/>
+    <col min="2" max="2" width="2.140625" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.28515625" style="1" customWidth="1"/>
+    <col min="10" max="14" width="11.28515625" style="1" customWidth="1"/>
+    <col min="15" max="17" width="11.28515625" customWidth="1"/>
+    <col min="18" max="18" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="3:18" ht="15" customHeight="1">
       <c r="D1" s="57" t="s">
         <v>575</v>
       </c>
@@ -11142,7 +11170,7 @@
       <c r="M1"/>
       <c r="N1"/>
     </row>
-    <row r="2" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="3:18">
       <c r="D2" s="57"/>
       <c r="E2" s="57"/>
       <c r="H2" s="57"/>
@@ -11153,7 +11181,7 @@
       <c r="M2"/>
       <c r="N2"/>
     </row>
-    <row r="3" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:18" ht="15" customHeight="1">
       <c r="D3" s="63"/>
       <c r="E3" s="63"/>
       <c r="F3" s="46"/>
@@ -11169,7 +11197,7 @@
       </c>
       <c r="R3" s="56"/>
     </row>
-    <row r="4" spans="3:18" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="3:18" ht="18.75">
       <c r="C4" s="62" t="s">
         <v>271</v>
       </c>
@@ -11197,7 +11225,7 @@
       <c r="Q4" s="56"/>
       <c r="R4" s="56"/>
     </row>
-    <row r="5" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:18">
       <c r="F5" s="29" t="s">
         <v>285</v>
       </c>
@@ -11208,7 +11236,7 @@
       <c r="Q5" s="56"/>
       <c r="R5" s="56"/>
     </row>
-    <row r="6" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:18">
       <c r="D6" s="60" t="s">
         <v>576</v>
       </c>
@@ -11224,7 +11252,7 @@
       <c r="Q6" s="22"/>
       <c r="R6" s="22"/>
     </row>
-    <row r="7" spans="3:18" s="2" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:18" s="2" customFormat="1" ht="38.25">
       <c r="C7" s="9" t="s">
         <v>3</v>
       </c>
@@ -11274,7 +11302,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="8" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:18">
       <c r="C8" s="3" t="s">
         <v>15</v>
       </c>
@@ -11325,7 +11353,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="9" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:18">
       <c r="C9" s="3" t="s">
         <v>16</v>
       </c>
@@ -11376,7 +11404,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="10" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:18">
       <c r="C10" s="3" t="s">
         <v>17</v>
       </c>
@@ -11427,7 +11455,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="11" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:18">
       <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
@@ -11478,7 +11506,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="12" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:18">
       <c r="C12" s="3" t="s">
         <v>19</v>
       </c>
@@ -11529,7 +11557,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="13" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:18">
       <c r="C13" s="3" t="s">
         <v>20</v>
       </c>
@@ -11580,7 +11608,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="14" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:18">
       <c r="C14" s="3" t="s">
         <v>21</v>
       </c>
@@ -11631,7 +11659,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="15" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:18">
       <c r="C15" s="3" t="s">
         <v>22</v>
       </c>
@@ -11682,7 +11710,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="16" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:18">
       <c r="C16" s="3" t="s">
         <v>23</v>
       </c>
@@ -11733,7 +11761,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="17" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:18">
       <c r="C17" s="3" t="s">
         <v>24</v>
       </c>
@@ -11784,7 +11812,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="18" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:18">
       <c r="C18" s="3" t="s">
         <v>25</v>
       </c>
@@ -11835,7 +11863,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="19" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:18">
       <c r="C19" s="3" t="s">
         <v>26</v>
       </c>
@@ -11886,7 +11914,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="20" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:18">
       <c r="C20" s="3" t="s">
         <v>27</v>
       </c>
@@ -11937,7 +11965,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="21" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:18">
       <c r="C21" s="3" t="s">
         <v>28</v>
       </c>
@@ -11988,7 +12016,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="22" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:18">
       <c r="C22" s="3" t="s">
         <v>29</v>
       </c>
@@ -12039,7 +12067,7 @@
         <v>35100</v>
       </c>
     </row>
-    <row r="23" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:18">
       <c r="C23" s="3" t="s">
         <v>30</v>
       </c>
@@ -12090,7 +12118,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="24" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:18">
       <c r="C24" s="3" t="s">
         <v>31</v>
       </c>
@@ -12141,7 +12169,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="25" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:18">
       <c r="C25" s="3" t="s">
         <v>32</v>
       </c>
@@ -12192,7 +12220,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="26" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:18">
       <c r="C26" s="3" t="s">
         <v>33</v>
       </c>
@@ -12243,7 +12271,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="27" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:18">
       <c r="C27" s="3" t="s">
         <v>34</v>
       </c>
@@ -12294,7 +12322,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="28" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:18">
       <c r="C28" s="3" t="s">
         <v>35</v>
       </c>
@@ -12345,7 +12373,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="29" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:18">
       <c r="C29" s="3" t="s">
         <v>36</v>
       </c>
@@ -12394,7 +12422,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="30" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:18">
       <c r="C30" s="3" t="s">
         <v>37</v>
       </c>
@@ -12445,7 +12473,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="31" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:18">
       <c r="C31" s="3" t="s">
         <v>38</v>
       </c>
@@ -12496,7 +12524,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="32" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:18">
       <c r="C32" s="3" t="s">
         <v>39</v>
       </c>
@@ -12547,7 +12575,7 @@
         <v>37800</v>
       </c>
     </row>
-    <row r="33" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:18">
       <c r="C33" s="3" t="s">
         <v>40</v>
       </c>
@@ -12598,7 +12626,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="34" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:18">
       <c r="C34" s="3" t="s">
         <v>41</v>
       </c>
@@ -12649,7 +12677,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="35" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:18">
       <c r="C35" s="3" t="s">
         <v>42</v>
       </c>
@@ -12700,7 +12728,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="36" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:18">
       <c r="C36" s="3" t="s">
         <v>43</v>
       </c>
@@ -12751,7 +12779,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="37" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:18">
       <c r="C37" s="3" t="s">
         <v>44</v>
       </c>
@@ -12802,7 +12830,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="38" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:18">
       <c r="C38" s="3" t="s">
         <v>45</v>
       </c>
@@ -12853,7 +12881,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="39" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:18">
       <c r="C39" s="3" t="s">
         <v>46</v>
       </c>
@@ -12904,7 +12932,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="40" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:18">
       <c r="C40" s="3" t="s">
         <v>47</v>
       </c>
@@ -12955,7 +12983,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="41" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:18">
       <c r="C41" s="3" t="s">
         <v>48</v>
       </c>
@@ -13006,7 +13034,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="42" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="42" spans="3:18">
       <c r="C42" s="3" t="s">
         <v>49</v>
       </c>
@@ -13057,7 +13085,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="43" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="43" spans="3:18">
       <c r="C43" s="3" t="s">
         <v>50</v>
       </c>
@@ -13108,7 +13136,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="44" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:18">
       <c r="C44" s="3" t="s">
         <v>51</v>
       </c>
@@ -13159,7 +13187,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="45" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="45" spans="3:18">
       <c r="C45" s="3" t="s">
         <v>52</v>
       </c>
@@ -13210,7 +13238,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="46" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:18">
       <c r="C46" s="3" t="s">
         <v>53</v>
       </c>
@@ -13259,7 +13287,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="47" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="47" spans="3:18">
       <c r="C47" s="3" t="s">
         <v>54</v>
       </c>
@@ -13310,7 +13338,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="48" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="48" spans="3:18">
       <c r="C48" s="3" t="s">
         <v>55</v>
       </c>
@@ -13361,7 +13389,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="49" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:18">
       <c r="C49" s="3" t="s">
         <v>56</v>
       </c>
@@ -13412,7 +13440,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="50" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:18">
       <c r="C50" s="3" t="s">
         <v>57</v>
       </c>
@@ -13463,7 +13491,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="51" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:18">
       <c r="C51" s="3" t="s">
         <v>58</v>
       </c>
@@ -13514,7 +13542,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="52" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:18">
       <c r="C52" s="3" t="s">
         <v>59</v>
       </c>
@@ -13565,7 +13593,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="53" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:18">
       <c r="C53" s="3" t="s">
         <v>60</v>
       </c>
@@ -13616,7 +13644,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="54" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:18">
       <c r="C54" s="3" t="s">
         <v>61</v>
       </c>
@@ -13667,7 +13695,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="55" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:18">
       <c r="C55" s="3" t="s">
         <v>62</v>
       </c>
@@ -13716,7 +13744,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="56" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="56" spans="3:18">
       <c r="C56" s="3" t="s">
         <v>63</v>
       </c>
@@ -13767,7 +13795,7 @@
         <v>37800</v>
       </c>
     </row>
-    <row r="57" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:18">
       <c r="C57" s="3" t="s">
         <v>64</v>
       </c>
@@ -13818,7 +13846,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="58" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:18">
       <c r="C58" s="3" t="s">
         <v>65</v>
       </c>
@@ -13869,7 +13897,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="59" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="59" spans="3:18">
       <c r="C59" s="3" t="s">
         <v>66</v>
       </c>
@@ -13920,7 +13948,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="60" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="60" spans="3:18">
       <c r="C60" s="3" t="s">
         <v>67</v>
       </c>
@@ -13971,7 +13999,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="61" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="61" spans="3:18">
       <c r="C61" s="3" t="s">
         <v>68</v>
       </c>
@@ -14022,7 +14050,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="62" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="62" spans="3:18">
       <c r="C62" s="3" t="s">
         <v>69</v>
       </c>
@@ -14073,7 +14101,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="63" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="63" spans="3:18">
       <c r="C63" s="3" t="s">
         <v>70</v>
       </c>
@@ -14124,7 +14152,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="64" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="64" spans="3:18">
       <c r="C64" s="3" t="s">
         <v>71</v>
       </c>
@@ -14175,7 +14203,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="65" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="65" spans="3:18">
       <c r="C65" s="3" t="s">
         <v>72</v>
       </c>
@@ -14226,7 +14254,7 @@
         <v>35100</v>
       </c>
     </row>
-    <row r="66" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="66" spans="3:18">
       <c r="C66" s="3" t="s">
         <v>73</v>
       </c>
@@ -14277,7 +14305,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="67" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="67" spans="3:18">
       <c r="C67" s="3" t="s">
         <v>74</v>
       </c>
@@ -14328,7 +14356,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="68" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="68" spans="3:18">
       <c r="C68" s="3" t="s">
         <v>75</v>
       </c>
@@ -14379,7 +14407,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="69" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="69" spans="3:18">
       <c r="C69" s="3" t="s">
         <v>76</v>
       </c>
@@ -14430,7 +14458,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="70" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="70" spans="3:18">
       <c r="C70" s="3" t="s">
         <v>77</v>
       </c>
@@ -14481,7 +14509,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="71" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="71" spans="3:18">
       <c r="C71" s="3" t="s">
         <v>78</v>
       </c>
@@ -14532,7 +14560,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="72" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="72" spans="3:18">
       <c r="C72" s="3" t="s">
         <v>79</v>
       </c>
@@ -14583,7 +14611,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="73" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="73" spans="3:18">
       <c r="C73" s="3" t="s">
         <v>80</v>
       </c>
@@ -14634,7 +14662,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="74" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="74" spans="3:18">
       <c r="C74" s="3" t="s">
         <v>81</v>
       </c>
@@ -14685,7 +14713,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="75" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="75" spans="3:18">
       <c r="C75" s="3" t="s">
         <v>82</v>
       </c>
@@ -14736,7 +14764,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="76" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="76" spans="3:18">
       <c r="C76" s="3" t="s">
         <v>83</v>
       </c>
@@ -14787,7 +14815,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="77" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="77" spans="3:18">
       <c r="C77" s="3" t="s">
         <v>84</v>
       </c>
@@ -14838,7 +14866,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="78" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="78" spans="3:18">
       <c r="C78" s="3" t="s">
         <v>85</v>
       </c>
@@ -14889,7 +14917,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="79" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="79" spans="3:18">
       <c r="C79" s="3" t="s">
         <v>86</v>
       </c>
@@ -14940,7 +14968,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="80" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="80" spans="3:18">
       <c r="C80" s="3" t="s">
         <v>87</v>
       </c>
@@ -14991,7 +15019,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="81" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="81" spans="3:18">
       <c r="C81" s="3" t="s">
         <v>88</v>
       </c>
@@ -15042,7 +15070,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="82" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="82" spans="3:18">
       <c r="C82" s="3" t="s">
         <v>89</v>
       </c>
@@ -15093,7 +15121,7 @@
         <v>37800</v>
       </c>
     </row>
-    <row r="83" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="83" spans="3:18">
       <c r="C83" s="3" t="s">
         <v>90</v>
       </c>
@@ -15144,7 +15172,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="84" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="84" spans="3:18">
       <c r="C84" s="3" t="s">
         <v>91</v>
       </c>
@@ -15195,7 +15223,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="85" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="85" spans="3:18">
       <c r="C85" s="3" t="s">
         <v>92</v>
       </c>
@@ -15246,7 +15274,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="86" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="86" spans="3:18">
       <c r="C86" s="3" t="s">
         <v>93</v>
       </c>
@@ -15297,7 +15325,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="87" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="87" spans="3:18">
       <c r="C87" s="3" t="s">
         <v>94</v>
       </c>
@@ -15348,7 +15376,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="88" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="88" spans="3:18">
       <c r="C88" s="3" t="s">
         <v>95</v>
       </c>
@@ -15399,7 +15427,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="89" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="89" spans="3:18">
       <c r="C89" s="3" t="s">
         <v>96</v>
       </c>
@@ -15450,7 +15478,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="90" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="90" spans="3:18">
       <c r="C90" s="3" t="s">
         <v>97</v>
       </c>
@@ -15501,7 +15529,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="91" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="91" spans="3:18">
       <c r="C91" s="3" t="s">
         <v>98</v>
       </c>
@@ -15552,7 +15580,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="92" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="92" spans="3:18">
       <c r="C92" s="3" t="s">
         <v>99</v>
       </c>
@@ -15603,7 +15631,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="93" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="93" spans="3:18">
       <c r="C93" s="3" t="s">
         <v>100</v>
       </c>
@@ -15654,7 +15682,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="94" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="94" spans="3:18">
       <c r="C94" s="3" t="s">
         <v>101</v>
       </c>
@@ -15705,7 +15733,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="95" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="95" spans="3:18">
       <c r="C95" s="3" t="s">
         <v>102</v>
       </c>
@@ -15756,7 +15784,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="96" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="96" spans="3:18">
       <c r="C96" s="3" t="s">
         <v>103</v>
       </c>
@@ -15807,7 +15835,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="97" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="97" spans="3:18">
       <c r="C97" s="3" t="s">
         <v>104</v>
       </c>
@@ -15858,7 +15886,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="98" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="98" spans="3:18">
       <c r="C98" s="3" t="s">
         <v>105</v>
       </c>
@@ -15909,7 +15937,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="99" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="99" spans="3:18">
       <c r="C99" s="3" t="s">
         <v>106</v>
       </c>
@@ -15960,7 +15988,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="100" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="100" spans="3:18">
       <c r="C100" s="3" t="s">
         <v>107</v>
       </c>
@@ -16011,7 +16039,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="101" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="101" spans="3:18">
       <c r="C101" s="3" t="s">
         <v>108</v>
       </c>
@@ -16062,7 +16090,7 @@
         <v>35100</v>
       </c>
     </row>
-    <row r="102" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="102" spans="3:18">
       <c r="C102" s="3" t="s">
         <v>109</v>
       </c>
@@ -16113,7 +16141,7 @@
         <v>35100</v>
       </c>
     </row>
-    <row r="103" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="103" spans="3:18">
       <c r="C103" s="3" t="s">
         <v>110</v>
       </c>
@@ -16164,7 +16192,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="104" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="104" spans="3:18">
       <c r="C104" s="3" t="s">
         <v>111</v>
       </c>
@@ -16215,7 +16243,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="105" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="105" spans="3:18">
       <c r="C105" s="3" t="s">
         <v>112</v>
       </c>
@@ -16266,7 +16294,7 @@
         <v>37800</v>
       </c>
     </row>
-    <row r="106" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="106" spans="3:18">
       <c r="C106" s="3" t="s">
         <v>113</v>
       </c>
@@ -16317,7 +16345,7 @@
         <v>35100</v>
       </c>
     </row>
-    <row r="107" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="107" spans="3:18">
       <c r="C107" s="3" t="s">
         <v>114</v>
       </c>
@@ -16368,7 +16396,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="108" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="108" spans="3:18">
       <c r="C108" s="3" t="s">
         <v>115</v>
       </c>
@@ -16419,7 +16447,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="109" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="109" spans="3:18">
       <c r="C109" s="3" t="s">
         <v>116</v>
       </c>
@@ -16470,7 +16498,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="110" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="110" spans="3:18">
       <c r="C110" s="3" t="s">
         <v>117</v>
       </c>
@@ -16521,7 +16549,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="111" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="111" spans="3:18">
       <c r="C111" s="3" t="s">
         <v>118</v>
       </c>
@@ -16572,7 +16600,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="112" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="112" spans="3:18">
       <c r="C112" s="3" t="s">
         <v>119</v>
       </c>
@@ -16623,7 +16651,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="113" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="113" spans="3:18">
       <c r="C113" s="3" t="s">
         <v>120</v>
       </c>
@@ -16674,7 +16702,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="114" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="114" spans="3:18">
       <c r="C114" s="3" t="s">
         <v>121</v>
       </c>
@@ -16725,7 +16753,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="115" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="115" spans="3:18">
       <c r="C115" s="3" t="s">
         <v>122</v>
       </c>
@@ -16776,7 +16804,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="116" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="116" spans="3:18">
       <c r="C116" s="3" t="s">
         <v>123</v>
       </c>
@@ -16827,7 +16855,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="117" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="117" spans="3:18">
       <c r="C117" s="3" t="s">
         <v>124</v>
       </c>
@@ -16878,7 +16906,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="118" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="118" spans="3:18">
       <c r="C118" s="3" t="s">
         <v>125</v>
       </c>
@@ -16929,7 +16957,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="119" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="119" spans="3:18">
       <c r="C119" s="3" t="s">
         <v>126</v>
       </c>
@@ -16980,7 +17008,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="120" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="120" spans="3:18">
       <c r="C120" s="3" t="s">
         <v>127</v>
       </c>
@@ -17031,7 +17059,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="121" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="121" spans="3:18">
       <c r="C121" s="3" t="s">
         <v>128</v>
       </c>
@@ -17082,7 +17110,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="122" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="122" spans="3:18">
       <c r="C122" s="3" t="s">
         <v>129</v>
       </c>
@@ -17133,7 +17161,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="123" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="123" spans="3:18">
       <c r="C123" s="3" t="s">
         <v>130</v>
       </c>
@@ -17184,7 +17212,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="124" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="124" spans="3:18">
       <c r="C124" s="3" t="s">
         <v>131</v>
       </c>
@@ -17235,7 +17263,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="125" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="125" spans="3:18">
       <c r="C125" s="3" t="s">
         <v>132</v>
       </c>
@@ -17286,7 +17314,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="126" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="126" spans="3:18">
       <c r="C126" s="3" t="s">
         <v>133</v>
       </c>
@@ -17337,7 +17365,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="127" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="127" spans="3:18">
       <c r="C127" s="3" t="s">
         <v>134</v>
       </c>
@@ -17388,7 +17416,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="128" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="128" spans="3:18">
       <c r="C128" s="3" t="s">
         <v>135</v>
       </c>
@@ -17439,7 +17467,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="129" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="129" spans="3:18">
       <c r="C129" s="3" t="s">
         <v>136</v>
       </c>
@@ -17490,7 +17518,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="130" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="130" spans="3:18">
       <c r="C130" s="3" t="s">
         <v>137</v>
       </c>
@@ -17541,7 +17569,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="131" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="131" spans="3:18">
       <c r="C131" s="3" t="s">
         <v>138</v>
       </c>
@@ -17592,7 +17620,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="132" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="132" spans="3:18">
       <c r="C132" s="3" t="s">
         <v>139</v>
       </c>
@@ -17643,7 +17671,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="133" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="133" spans="3:18">
       <c r="C133" s="3" t="s">
         <v>140</v>
       </c>
@@ -17694,7 +17722,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="134" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="134" spans="3:18">
       <c r="C134" s="3" t="s">
         <v>141</v>
       </c>
@@ -17745,7 +17773,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="135" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="135" spans="3:18">
       <c r="C135" s="3" t="s">
         <v>142</v>
       </c>
@@ -17796,7 +17824,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="136" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="136" spans="3:18">
       <c r="C136" s="3" t="s">
         <v>143</v>
       </c>
@@ -17847,7 +17875,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="137" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="137" spans="3:18">
       <c r="C137" s="3" t="s">
         <v>144</v>
       </c>
@@ -17898,7 +17926,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="138" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="138" spans="3:18">
       <c r="C138" s="3" t="s">
         <v>145</v>
       </c>
@@ -17949,7 +17977,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="139" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="139" spans="3:18">
       <c r="C139" s="3" t="s">
         <v>146</v>
       </c>
@@ -18000,7 +18028,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="140" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="140" spans="3:18">
       <c r="C140" s="3" t="s">
         <v>147</v>
       </c>
@@ -18051,7 +18079,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="141" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="141" spans="3:18">
       <c r="C141" s="3" t="s">
         <v>148</v>
       </c>
@@ -18102,7 +18130,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="142" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="142" spans="3:18">
       <c r="C142" s="3" t="s">
         <v>149</v>
       </c>
@@ -18153,7 +18181,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="143" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="143" spans="3:18">
       <c r="C143" s="3" t="s">
         <v>150</v>
       </c>
@@ -18204,7 +18232,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="144" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="144" spans="3:18">
       <c r="C144" s="3" t="s">
         <v>151</v>
       </c>
@@ -18255,7 +18283,7 @@
         <v>10800</v>
       </c>
     </row>
-    <row r="145" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="145" spans="3:18">
       <c r="C145" s="3" t="s">
         <v>152</v>
       </c>
@@ -18306,7 +18334,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="146" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="146" spans="3:18">
       <c r="C146" s="3" t="s">
         <v>153</v>
       </c>
@@ -18357,7 +18385,7 @@
         <v>37800</v>
       </c>
     </row>
-    <row r="147" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="147" spans="3:18">
       <c r="C147" s="3" t="s">
         <v>154</v>
       </c>
@@ -18408,7 +18436,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="148" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="148" spans="3:18">
       <c r="C148" s="3" t="s">
         <v>155</v>
       </c>
@@ -18459,7 +18487,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="149" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="149" spans="3:18">
       <c r="C149" s="3" t="s">
         <v>156</v>
       </c>
@@ -18510,7 +18538,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="150" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="150" spans="3:18">
       <c r="C150" s="3" t="s">
         <v>157</v>
       </c>
@@ -18561,7 +18589,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="151" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="151" spans="3:18">
       <c r="C151" s="3" t="s">
         <v>158</v>
       </c>
@@ -18612,7 +18640,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="152" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="152" spans="3:18">
       <c r="C152" s="3" t="s">
         <v>159</v>
       </c>
@@ -18663,7 +18691,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="153" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="153" spans="3:18">
       <c r="C153" s="3" t="s">
         <v>160</v>
       </c>
@@ -18714,7 +18742,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="154" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="154" spans="3:18">
       <c r="C154" s="3" t="s">
         <v>161</v>
       </c>
@@ -18765,7 +18793,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="155" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="155" spans="3:18">
       <c r="C155" s="3" t="s">
         <v>162</v>
       </c>
@@ -18816,7 +18844,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="156" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="156" spans="3:18">
       <c r="C156" s="3" t="s">
         <v>163</v>
       </c>
@@ -18867,7 +18895,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="157" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="157" spans="3:18">
       <c r="C157" s="3" t="s">
         <v>164</v>
       </c>
@@ -18918,7 +18946,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="158" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="158" spans="3:18">
       <c r="C158" s="3" t="s">
         <v>165</v>
       </c>
@@ -18969,7 +18997,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="159" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="159" spans="3:18">
       <c r="C159" s="3" t="s">
         <v>166</v>
       </c>
@@ -19020,7 +19048,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="160" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="160" spans="3:18">
       <c r="C160" s="3" t="s">
         <v>167</v>
       </c>
@@ -19071,7 +19099,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="161" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="161" spans="3:18">
       <c r="C161" s="3" t="s">
         <v>168</v>
       </c>
@@ -19122,7 +19150,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="162" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="162" spans="3:18">
       <c r="C162" s="3" t="s">
         <v>169</v>
       </c>
@@ -19173,7 +19201,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="163" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="163" spans="3:18">
       <c r="C163" s="3" t="s">
         <v>170</v>
       </c>
@@ -19224,7 +19252,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="164" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="164" spans="3:18">
       <c r="C164" s="3" t="s">
         <v>171</v>
       </c>
@@ -19275,7 +19303,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="165" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="165" spans="3:18">
       <c r="C165" s="3" t="s">
         <v>172</v>
       </c>
@@ -19326,7 +19354,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="166" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="166" spans="3:18">
       <c r="C166" s="3" t="s">
         <v>173</v>
       </c>
@@ -19377,7 +19405,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="167" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="167" spans="3:18">
       <c r="C167" s="3" t="s">
         <v>174</v>
       </c>
@@ -19428,7 +19456,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="168" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="168" spans="3:18">
       <c r="C168" s="3" t="s">
         <v>175</v>
       </c>
@@ -19479,7 +19507,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="169" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="169" spans="3:18">
       <c r="C169" s="3" t="s">
         <v>176</v>
       </c>
@@ -19530,7 +19558,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="170" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="170" spans="3:18">
       <c r="C170" s="3" t="s">
         <v>177</v>
       </c>
@@ -19581,7 +19609,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="171" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="171" spans="3:18">
       <c r="C171" s="3" t="s">
         <v>178</v>
       </c>
@@ -19632,7 +19660,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="172" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="172" spans="3:18">
       <c r="C172" s="3" t="s">
         <v>179</v>
       </c>
@@ -19683,7 +19711,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="173" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="173" spans="3:18">
       <c r="C173" s="3" t="s">
         <v>180</v>
       </c>
@@ -19734,7 +19762,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="174" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="174" spans="3:18">
       <c r="C174" s="3" t="s">
         <v>181</v>
       </c>
@@ -19785,7 +19813,7 @@
         <v>10800</v>
       </c>
     </row>
-    <row r="175" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="175" spans="3:18">
       <c r="C175" s="3" t="s">
         <v>182</v>
       </c>
@@ -19836,7 +19864,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="176" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="176" spans="3:18">
       <c r="C176" s="3" t="s">
         <v>183</v>
       </c>
@@ -19887,7 +19915,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="177" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="177" spans="3:18">
       <c r="C177" s="3" t="s">
         <v>184</v>
       </c>
@@ -19938,7 +19966,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="178" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="178" spans="3:18">
       <c r="C178" s="3" t="s">
         <v>185</v>
       </c>
@@ -19989,7 +20017,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="179" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="179" spans="3:18">
       <c r="C179" s="3" t="s">
         <v>186</v>
       </c>
@@ -20040,7 +20068,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="180" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="180" spans="3:18">
       <c r="C180" s="3" t="s">
         <v>187</v>
       </c>
@@ -20091,7 +20119,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="181" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="181" spans="3:18">
       <c r="C181" s="3" t="s">
         <v>188</v>
       </c>
@@ -20142,7 +20170,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="182" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="182" spans="3:18">
       <c r="C182" s="3" t="s">
         <v>189</v>
       </c>
@@ -20193,7 +20221,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="183" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="183" spans="3:18">
       <c r="C183" s="3" t="s">
         <v>190</v>
       </c>
@@ -20244,7 +20272,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="184" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="184" spans="3:18">
       <c r="C184" s="3" t="s">
         <v>191</v>
       </c>
@@ -20295,7 +20323,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="185" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="185" spans="3:18">
       <c r="C185" s="3" t="s">
         <v>192</v>
       </c>
@@ -20346,7 +20374,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="186" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="186" spans="3:18">
       <c r="C186" s="3" t="s">
         <v>193</v>
       </c>
@@ -20397,7 +20425,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="187" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="187" spans="3:18">
       <c r="C187" s="3" t="s">
         <v>194</v>
       </c>
@@ -20448,7 +20476,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="188" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="188" spans="3:18">
       <c r="C188" s="3" t="s">
         <v>195</v>
       </c>
@@ -20499,7 +20527,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="189" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="189" spans="3:18">
       <c r="C189" s="3" t="s">
         <v>196</v>
       </c>
@@ -20550,7 +20578,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="190" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="190" spans="3:18">
       <c r="C190" s="3" t="s">
         <v>197</v>
       </c>
@@ -20601,7 +20629,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="191" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="191" spans="3:18">
       <c r="C191" s="3" t="s">
         <v>198</v>
       </c>
@@ -20652,7 +20680,7 @@
         <v>13500</v>
       </c>
     </row>
-    <row r="192" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="192" spans="3:18">
       <c r="C192" s="3" t="s">
         <v>199</v>
       </c>
@@ -20703,7 +20731,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="193" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="193" spans="3:18">
       <c r="C193" s="3" t="s">
         <v>200</v>
       </c>
@@ -20754,7 +20782,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="194" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="194" spans="3:18">
       <c r="C194" s="3" t="s">
         <v>201</v>
       </c>
@@ -20805,7 +20833,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="195" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="195" spans="3:18">
       <c r="C195" s="3" t="s">
         <v>202</v>
       </c>
@@ -20856,7 +20884,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="196" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="196" spans="3:18">
       <c r="C196" s="3" t="s">
         <v>203</v>
       </c>
@@ -20907,7 +20935,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="197" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="197" spans="3:18">
       <c r="C197" s="3" t="s">
         <v>204</v>
       </c>
@@ -20958,7 +20986,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="198" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="198" spans="3:18">
       <c r="C198" s="3" t="s">
         <v>205</v>
       </c>
@@ -21009,7 +21037,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="199" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="199" spans="3:18">
       <c r="C199" s="3" t="s">
         <v>206</v>
       </c>
@@ -21060,7 +21088,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="200" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="200" spans="3:18">
       <c r="C200" s="3" t="s">
         <v>207</v>
       </c>
@@ -21111,7 +21139,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="201" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="201" spans="3:18">
       <c r="C201" s="3" t="s">
         <v>208</v>
       </c>
@@ -21162,7 +21190,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="202" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="202" spans="3:18">
       <c r="C202" s="3" t="s">
         <v>209</v>
       </c>
@@ -21213,7 +21241,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="203" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="203" spans="3:18">
       <c r="C203" s="3" t="s">
         <v>210</v>
       </c>
@@ -21264,7 +21292,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="204" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="204" spans="3:18">
       <c r="C204" s="3" t="s">
         <v>211</v>
       </c>
@@ -21315,7 +21343,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="205" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="205" spans="3:18">
       <c r="C205" s="3" t="s">
         <v>212</v>
       </c>
@@ -21366,7 +21394,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="206" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="206" spans="3:18">
       <c r="C206" s="3" t="s">
         <v>213</v>
       </c>
@@ -21417,7 +21445,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="207" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="207" spans="3:18">
       <c r="C207" s="3" t="s">
         <v>214</v>
       </c>
@@ -21468,7 +21496,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="208" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="208" spans="3:18">
       <c r="C208" s="3" t="s">
         <v>215</v>
       </c>
@@ -21519,7 +21547,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="209" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="209" spans="3:18">
       <c r="C209" s="3" t="s">
         <v>216</v>
       </c>
@@ -21570,7 +21598,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="210" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="210" spans="3:18">
       <c r="C210" s="3" t="s">
         <v>217</v>
       </c>
@@ -21621,7 +21649,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="211" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="211" spans="3:18">
       <c r="C211" s="3" t="s">
         <v>218</v>
       </c>
@@ -21672,7 +21700,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="212" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="212" spans="3:18">
       <c r="C212" s="3" t="s">
         <v>219</v>
       </c>
@@ -21723,7 +21751,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="213" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="213" spans="3:18">
       <c r="C213" s="3" t="s">
         <v>220</v>
       </c>
@@ -21774,7 +21802,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="214" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="214" spans="3:18">
       <c r="C214" s="3" t="s">
         <v>221</v>
       </c>
@@ -21825,7 +21853,7 @@
         <v>13500</v>
       </c>
     </row>
-    <row r="215" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="215" spans="3:18">
       <c r="C215" s="3" t="s">
         <v>222</v>
       </c>
@@ -21876,7 +21904,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="216" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="216" spans="3:18">
       <c r="C216" s="3" t="s">
         <v>223</v>
       </c>
@@ -21927,7 +21955,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="217" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="217" spans="3:18">
       <c r="C217" s="3" t="s">
         <v>224</v>
       </c>
@@ -21978,7 +22006,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="218" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="218" spans="3:18">
       <c r="C218" s="3" t="s">
         <v>225</v>
       </c>
@@ -22029,7 +22057,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="219" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="219" spans="3:18">
       <c r="C219" s="3" t="s">
         <v>226</v>
       </c>
@@ -22080,7 +22108,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="220" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="220" spans="3:18">
       <c r="C220" s="3" t="s">
         <v>227</v>
       </c>
@@ -22131,7 +22159,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="221" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="221" spans="3:18">
       <c r="C221" s="3" t="s">
         <v>228</v>
       </c>
@@ -22182,7 +22210,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="222" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="222" spans="3:18">
       <c r="C222" s="3" t="s">
         <v>229</v>
       </c>
@@ -22233,7 +22261,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="223" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="223" spans="3:18">
       <c r="C223" s="3" t="s">
         <v>230</v>
       </c>
@@ -22284,7 +22312,7 @@
         <v>35100</v>
       </c>
     </row>
-    <row r="224" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="224" spans="3:18">
       <c r="C224" s="3" t="s">
         <v>231</v>
       </c>
@@ -22335,7 +22363,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="225" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="225" spans="3:18">
       <c r="C225" s="3" t="s">
         <v>232</v>
       </c>
@@ -22386,7 +22414,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="226" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="226" spans="3:18">
       <c r="C226" s="3" t="s">
         <v>233</v>
       </c>
@@ -22437,7 +22465,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="227" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="227" spans="3:18">
       <c r="C227" s="3" t="s">
         <v>234</v>
       </c>
@@ -22488,7 +22516,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="228" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="228" spans="3:18">
       <c r="C228" s="3" t="s">
         <v>235</v>
       </c>
@@ -22539,7 +22567,7 @@
         <v>10800</v>
       </c>
     </row>
-    <row r="229" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="229" spans="3:18">
       <c r="C229" s="3" t="s">
         <v>236</v>
       </c>
@@ -22590,7 +22618,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="230" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="230" spans="3:18">
       <c r="C230" s="3" t="s">
         <v>237</v>
       </c>
@@ -22641,7 +22669,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="231" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="231" spans="3:18">
       <c r="C231" s="3" t="s">
         <v>238</v>
       </c>
@@ -22692,7 +22720,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="232" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="232" spans="3:18">
       <c r="C232" s="3" t="s">
         <v>239</v>
       </c>
@@ -22743,7 +22771,7 @@
         <v>32400</v>
       </c>
     </row>
-    <row r="233" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="233" spans="3:18">
       <c r="C233" s="3" t="s">
         <v>240</v>
       </c>
@@ -22794,7 +22822,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="234" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="234" spans="3:18">
       <c r="C234" s="3" t="s">
         <v>241</v>
       </c>
@@ -22845,7 +22873,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="235" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="235" spans="3:18">
       <c r="C235" s="3" t="s">
         <v>242</v>
       </c>
@@ -22896,7 +22924,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="236" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="236" spans="3:18">
       <c r="C236" s="3" t="s">
         <v>243</v>
       </c>
@@ -22947,7 +22975,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="237" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="237" spans="3:18">
       <c r="C237" s="3" t="s">
         <v>244</v>
       </c>
@@ -22998,7 +23026,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="238" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="238" spans="3:18">
       <c r="C238" s="3" t="s">
         <v>245</v>
       </c>
@@ -23049,7 +23077,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="239" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="239" spans="3:18">
       <c r="C239" s="3" t="s">
         <v>246</v>
       </c>
@@ -23100,7 +23128,7 @@
         <v>35100</v>
       </c>
     </row>
-    <row r="240" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="240" spans="3:18">
       <c r="C240" s="3" t="s">
         <v>247</v>
       </c>
@@ -23151,7 +23179,7 @@
         <v>16200</v>
       </c>
     </row>
-    <row r="241" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="241" spans="3:18">
       <c r="C241" s="3" t="s">
         <v>248</v>
       </c>
@@ -23202,7 +23230,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="242" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="242" spans="3:18">
       <c r="C242" s="3" t="s">
         <v>249</v>
       </c>
@@ -23253,7 +23281,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="243" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="243" spans="3:18">
       <c r="C243" s="3" t="s">
         <v>250</v>
       </c>
@@ -23304,7 +23332,7 @@
         <v>13500</v>
       </c>
     </row>
-    <row r="244" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="244" spans="3:18">
       <c r="C244" s="3" t="s">
         <v>251</v>
       </c>
@@ -23355,7 +23383,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="245" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="245" spans="3:18">
       <c r="C245" s="3" t="s">
         <v>252</v>
       </c>
@@ -23406,7 +23434,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="246" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="246" spans="3:18">
       <c r="C246" s="3" t="s">
         <v>253</v>
       </c>
@@ -23457,7 +23485,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="247" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="247" spans="3:18">
       <c r="C247" s="3" t="s">
         <v>254</v>
       </c>
@@ -23508,7 +23536,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="248" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="248" spans="3:18">
       <c r="C248" s="3" t="s">
         <v>255</v>
       </c>
@@ -23559,7 +23587,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="249" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="249" spans="3:18">
       <c r="C249" s="3" t="s">
         <v>256</v>
       </c>
@@ -23610,7 +23638,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="250" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="250" spans="3:18">
       <c r="C250" s="3" t="s">
         <v>257</v>
       </c>
@@ -23661,7 +23689,7 @@
         <v>18900</v>
       </c>
     </row>
-    <row r="251" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="251" spans="3:18">
       <c r="C251" s="3" t="s">
         <v>258</v>
       </c>
@@ -23712,7 +23740,7 @@
         <v>27000</v>
       </c>
     </row>
-    <row r="252" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="252" spans="3:18">
       <c r="C252" s="3" t="s">
         <v>259</v>
       </c>
@@ -23763,7 +23791,7 @@
         <v>24300</v>
       </c>
     </row>
-    <row r="253" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="253" spans="3:18">
       <c r="C253" s="3" t="s">
         <v>260</v>
       </c>
@@ -23814,7 +23842,7 @@
         <v>21600</v>
       </c>
     </row>
-    <row r="254" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="254" spans="3:18">
       <c r="C254" s="3" t="s">
         <v>261</v>
       </c>
@@ -23865,7 +23893,7 @@
         <v>29700</v>
       </c>
     </row>
-    <row r="255" spans="3:18" x14ac:dyDescent="0.3">
+    <row r="255" spans="3:18">
       <c r="C255" s="3" t="s">
         <v>262</v>
       </c>
@@ -23914,6 +23942,12 @@
       <c r="R255" s="45">
         <f t="shared" si="3"/>
         <v>16200</v>
+      </c>
+    </row>
+    <row r="257" spans="18:18">
+      <c r="R257" s="86">
+        <f>SUM(Total_Payment)</f>
+        <v>6021000</v>
       </c>
     </row>
   </sheetData>
@@ -23941,7 +23975,7 @@
       <formula>AND(_xlfn.ISFORMULA($J$4),$J$4=1535)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R8:R255">
+  <conditionalFormatting sqref="R8:R255 R257">
     <cfRule type="expression" dxfId="1" priority="5">
       <formula>AND(_xlfn.ISFORMULA(R8),R8=O8+P8+Q8)</formula>
     </cfRule>
@@ -23953,74 +23987,74 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M55"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="16.33203125" customWidth="1"/>
-    <col min="7" max="9" width="11.33203125" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" customWidth="1"/>
-    <col min="11" max="13" width="11.33203125" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="9" width="11.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" customWidth="1"/>
+    <col min="11" max="13" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+    <row r="1" spans="1:12" ht="15" customHeight="1">
+      <c r="A1" s="67" t="s">
         <v>585</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="D1" s="68" t="s">
+      <c r="B1" s="67"/>
+      <c r="D1" s="71" t="s">
         <v>587</v>
       </c>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="I1" s="68" t="s">
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="I1" s="71" t="s">
         <v>586</v>
       </c>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="66"/>
-      <c r="B2" s="66"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="67"/>
-      <c r="B3" s="67"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-    </row>
-    <row r="4" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="65" t="s">
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="67"/>
+      <c r="B2" s="67"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="81"/>
+      <c r="B3" s="81"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="71"/>
+    </row>
+    <row r="4" spans="1:12" ht="29.25" customHeight="1">
+      <c r="A4" s="80" t="s">
         <v>273</v>
       </c>
-      <c r="B4" s="65"/>
+      <c r="B4" s="80"/>
       <c r="C4" s="14"/>
       <c r="D4" s="16"/>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
     </row>
-    <row r="5" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="23.25" customHeight="1">
       <c r="A5" s="15" t="s">
         <v>263</v>
       </c>
@@ -24029,7 +24063,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="23.25" customHeight="1">
       <c r="A6" s="15" t="s">
         <v>264</v>
       </c>
@@ -24039,7 +24073,7 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="23.25" customHeight="1">
       <c r="A7" s="15" t="s">
         <v>265</v>
       </c>
@@ -24048,31 +24082,31 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" ht="12" customHeight="1">
       <c r="A8" s="17"/>
       <c r="B8" s="6"/>
     </row>
-    <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="66" t="s">
+    <row r="9" spans="1:12" ht="15" customHeight="1">
+      <c r="A9" s="67" t="s">
         <v>588</v>
       </c>
-      <c r="B9" s="66"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" s="66"/>
-      <c r="B10" s="66"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11" s="67"/>
-      <c r="B11" s="67"/>
-    </row>
-    <row r="12" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A12" s="65" t="s">
+      <c r="B9" s="67"/>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" s="67"/>
+      <c r="B10" s="67"/>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" s="81"/>
+      <c r="B11" s="81"/>
+    </row>
+    <row r="12" spans="1:12" ht="18.75">
+      <c r="A12" s="80" t="s">
         <v>274</v>
       </c>
-      <c r="B12" s="65"/>
-    </row>
-    <row r="13" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+      <c r="B12" s="80"/>
+    </row>
+    <row r="13" spans="1:12" ht="18.75">
       <c r="A13" s="15" t="s">
         <v>268</v>
       </c>
@@ -24081,7 +24115,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" ht="18.75">
       <c r="A14" s="15" t="s">
         <v>269</v>
       </c>
@@ -24090,7 +24124,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" ht="18.75">
       <c r="A15" s="15" t="s">
         <v>270</v>
       </c>
@@ -24099,12 +24133,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="73" t="s">
+    <row r="17" spans="1:13" ht="24.75" customHeight="1">
+      <c r="A17" s="84" t="s">
         <v>589</v>
       </c>
-      <c r="B17" s="73"/>
-      <c r="C17" s="74"/>
+      <c r="B17" s="84"/>
+      <c r="C17" s="85"/>
       <c r="D17" s="28" t="s">
         <v>275</v>
       </c>
@@ -24114,11 +24148,11 @@
       <c r="F17" s="28" t="s">
         <v>277</v>
       </c>
-      <c r="H17" s="73" t="s">
+      <c r="H17" s="84" t="s">
         <v>590</v>
       </c>
-      <c r="I17" s="73"/>
-      <c r="J17" s="74"/>
+      <c r="I17" s="84"/>
+      <c r="J17" s="85"/>
       <c r="K17" s="28" t="s">
         <v>275</v>
       </c>
@@ -24129,12 +24163,12 @@
         <v>277</v>
       </c>
     </row>
-    <row r="18" spans="1:13" s="19" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="69" t="s">
+    <row r="18" spans="1:13" s="19" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A18" s="70" t="s">
         <v>551</v>
       </c>
-      <c r="B18" s="70"/>
-      <c r="C18" s="71"/>
+      <c r="B18" s="82"/>
+      <c r="C18" s="83"/>
       <c r="D18" s="20">
         <f>COUNTIFS(Number_of_units__Semester_1,"&gt;4")</f>
         <v>47</v>
@@ -24147,11 +24181,11 @@
         <f>COUNTIFS(Number_of_units__Semester_3,"&gt;4")</f>
         <v>57</v>
       </c>
-      <c r="H18" s="72" t="s">
+      <c r="H18" s="69" t="s">
         <v>553</v>
       </c>
-      <c r="I18" s="72"/>
-      <c r="J18" s="69"/>
+      <c r="I18" s="69"/>
+      <c r="J18" s="70"/>
       <c r="K18" s="20">
         <f>COUNTIFS(Average_mark_Semester_1,"&lt;50")</f>
         <v>36</v>
@@ -24165,12 +24199,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:13" s="19" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="72" t="s">
+    <row r="19" spans="1:13" s="19" customFormat="1" ht="22.5" customHeight="1">
+      <c r="A19" s="69" t="s">
         <v>552</v>
       </c>
-      <c r="B19" s="72"/>
-      <c r="C19" s="69"/>
+      <c r="B19" s="69"/>
+      <c r="C19" s="70"/>
       <c r="D19" s="20">
         <f>COUNTIFS(Number_of_units__Semester_1,1)</f>
         <v>39</v>
@@ -24183,11 +24217,11 @@
         <f>COUNTIFS(Number_of_units__Semester_3,1)</f>
         <v>0</v>
       </c>
-      <c r="H19" s="72" t="s">
+      <c r="H19" s="69" t="s">
         <v>284</v>
       </c>
-      <c r="I19" s="72"/>
-      <c r="J19" s="69"/>
+      <c r="I19" s="69"/>
+      <c r="J19" s="70"/>
       <c r="K19" s="20">
         <f>COUNTIFS(Average_mark_Semester_1,"&lt;50",Course,"Accounting")</f>
         <v>9</v>
@@ -24201,7 +24235,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:13" s="19" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" s="19" customFormat="1" ht="22.5" customHeight="1">
       <c r="A20" s="25"/>
       <c r="B20" s="25"/>
       <c r="C20" s="25"/>
@@ -24209,50 +24243,50 @@
       <c r="E20" s="26"/>
       <c r="F20" s="26"/>
     </row>
-    <row r="21" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" ht="18.75" customHeight="1">
       <c r="A21" s="18"/>
       <c r="H21" s="27"/>
       <c r="I21" s="27"/>
       <c r="J21" s="27"/>
       <c r="K21" s="27"/>
     </row>
-    <row r="22" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" ht="18.75" customHeight="1">
       <c r="A22" s="18"/>
       <c r="H22" s="27"/>
       <c r="I22" s="27"/>
       <c r="J22" s="27"/>
       <c r="K22" s="27"/>
     </row>
-    <row r="23" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" ht="18.75" customHeight="1">
       <c r="A23" s="18"/>
-      <c r="B23" s="84" t="s">
+      <c r="B23" s="78" t="s">
         <v>592</v>
       </c>
-      <c r="C23" s="82" t="s">
+      <c r="C23" s="76" t="s">
         <v>591</v>
       </c>
-      <c r="D23" s="82"/>
-      <c r="E23" s="82"/>
-      <c r="G23" s="66" t="s">
+      <c r="D23" s="76"/>
+      <c r="E23" s="76"/>
+      <c r="G23" s="67" t="s">
         <v>580</v>
       </c>
-      <c r="H23" s="66"/>
-      <c r="I23" s="66"/>
-      <c r="J23" s="66"/>
-      <c r="K23" s="66"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B24" s="85"/>
-      <c r="C24" s="82"/>
-      <c r="D24" s="82"/>
-      <c r="E24" s="82"/>
-      <c r="G24" s="66"/>
-      <c r="H24" s="66"/>
-      <c r="I24" s="66"/>
-      <c r="J24" s="66"/>
-      <c r="K24" s="66"/>
-    </row>
-    <row r="25" spans="1:13" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="H23" s="67"/>
+      <c r="I23" s="67"/>
+      <c r="J23" s="67"/>
+      <c r="K23" s="67"/>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="B24" s="79"/>
+      <c r="C24" s="76"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="G24" s="67"/>
+      <c r="H24" s="67"/>
+      <c r="I24" s="67"/>
+      <c r="J24" s="67"/>
+      <c r="K24" s="67"/>
+    </row>
+    <row r="25" spans="1:13" ht="31.5">
       <c r="A25" s="44" t="s">
         <v>278</v>
       </c>
@@ -24273,7 +24307,7 @@
       <c r="I25" s="33"/>
       <c r="J25" s="33"/>
     </row>
-    <row r="26" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" ht="18.75">
       <c r="A26" s="15" t="s">
         <v>263</v>
       </c>
@@ -24295,7 +24329,7 @@
       </c>
       <c r="G26" s="7"/>
     </row>
-    <row r="27" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" ht="18.75">
       <c r="A27" s="15" t="s">
         <v>264</v>
       </c>
@@ -24316,7 +24350,7 @@
         <v>680400</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" ht="18.75">
       <c r="A28" s="15" t="s">
         <v>265</v>
       </c>
@@ -24337,48 +24371,48 @@
         <v>267300</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="141.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" ht="141.75" customHeight="1">
       <c r="A29" s="17"/>
       <c r="B29" s="32"/>
       <c r="C29" s="32"/>
       <c r="D29" s="32"/>
       <c r="E29" s="32"/>
     </row>
-    <row r="30" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H30" s="68" t="s">
+    <row r="30" spans="1:13" ht="31.5" customHeight="1">
+      <c r="H30" s="71" t="s">
         <v>582</v>
       </c>
-      <c r="I30" s="68"/>
-      <c r="J30" s="68"/>
-      <c r="K30" s="68"/>
-    </row>
-    <row r="31" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="78" t="s">
+      <c r="I30" s="71"/>
+      <c r="J30" s="71"/>
+      <c r="K30" s="71"/>
+    </row>
+    <row r="31" spans="1:13" ht="15" customHeight="1">
+      <c r="B31" s="72" t="s">
         <v>593</v>
       </c>
-      <c r="C31" s="79"/>
-      <c r="D31" s="79"/>
-      <c r="E31" s="82" t="s">
+      <c r="C31" s="73"/>
+      <c r="D31" s="73"/>
+      <c r="E31" s="76" t="s">
         <v>581</v>
       </c>
-      <c r="F31" s="83"/>
+      <c r="F31" s="77"/>
       <c r="H31" s="27"/>
       <c r="I31" s="27"/>
       <c r="J31" s="27"/>
       <c r="K31" s="27"/>
     </row>
-    <row r="32" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="80"/>
-      <c r="C32" s="81"/>
-      <c r="D32" s="81"/>
-      <c r="E32" s="82"/>
-      <c r="F32" s="83"/>
+    <row r="32" spans="1:13" ht="15" customHeight="1">
+      <c r="B32" s="74"/>
+      <c r="C32" s="75"/>
+      <c r="D32" s="75"/>
+      <c r="E32" s="76"/>
+      <c r="F32" s="77"/>
       <c r="H32" s="27"/>
       <c r="I32" s="27"/>
       <c r="J32" s="27"/>
       <c r="K32" s="27"/>
     </row>
-    <row r="33" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="31.5">
       <c r="A33" s="12" t="s">
         <v>286</v>
       </c>
@@ -24396,7 +24430,7 @@
       </c>
       <c r="F33" s="34"/>
     </row>
-    <row r="34" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" ht="18.75">
       <c r="A34" s="15" t="s">
         <v>275</v>
       </c>
@@ -24419,7 +24453,7 @@
       <c r="F34" s="35"/>
       <c r="G34" s="7"/>
     </row>
-    <row r="35" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" ht="18.75">
       <c r="A35" s="15" t="s">
         <v>276</v>
       </c>
@@ -24441,7 +24475,7 @@
       </c>
       <c r="F35" s="35"/>
     </row>
-    <row r="36" spans="1:7" ht="18" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="18.75">
       <c r="A36" s="15" t="s">
         <v>277</v>
       </c>
@@ -24463,7 +24497,7 @@
       </c>
       <c r="F36" s="35"/>
     </row>
-    <row r="37" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" ht="21.75" customHeight="1">
       <c r="A37" s="24" t="s">
         <v>283</v>
       </c>
@@ -24472,76 +24506,66 @@
       <c r="D37" s="13"/>
       <c r="E37" s="13"/>
     </row>
-    <row r="38" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="75" t="s">
+    <row r="38" spans="1:7" ht="15" customHeight="1">
+      <c r="A38" s="65" t="s">
         <v>583</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="76"/>
+    <row r="39" spans="1:7" ht="15" customHeight="1">
+      <c r="A39" s="66"/>
       <c r="B39" t="s">
         <v>594</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="76"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="76"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" s="76"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" s="77" t="s">
+    <row r="40" spans="1:7">
+      <c r="A40" s="66"/>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="66"/>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="66"/>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" s="68" t="s">
         <v>584</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" s="77"/>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A47" s="77"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="77"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="77"/>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" s="77"/>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="77"/>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="77"/>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="77"/>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" s="77"/>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" s="77"/>
+    <row r="46" spans="1:7">
+      <c r="A46" s="68"/>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47" s="68"/>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" s="68"/>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" s="68"/>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" s="68"/>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" s="68"/>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" s="68"/>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" s="68"/>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" s="68"/>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" s="68"/>
     </row>
   </sheetData>
-  <sortState ref="E6:E72">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E6:E72">
     <sortCondition ref="E6"/>
   </sortState>
   <mergeCells count="21">
-    <mergeCell ref="A38:A42"/>
-    <mergeCell ref="G23:K24"/>
-    <mergeCell ref="A45:A55"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="H30:K30"/>
-    <mergeCell ref="B31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C23:E24"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A9:B11"/>
     <mergeCell ref="I1:L3"/>
@@ -24553,6 +24577,16 @@
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="D1:G3"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A38:A42"/>
+    <mergeCell ref="G23:K24"/>
+    <mergeCell ref="A45:A55"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="H30:K30"/>
+    <mergeCell ref="B31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:E24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -24577,7 +24611,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{05C60535-1F16-4fd2-B633-F4F36F0B64E0}">
       <x14:sparklineGroups xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-        <x14:sparklineGroup displayEmptyCellsAs="gap">
+        <x14:sparklineGroup displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0200-000000000000}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>
@@ -24612,27 +24646,27 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A4:M37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="16.33203125" customWidth="1"/>
-    <col min="7" max="9" width="11.33203125" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" customWidth="1"/>
-    <col min="11" max="13" width="11.33203125" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="9" width="11.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" customWidth="1"/>
+    <col min="11" max="13" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>263</v>
       </c>
@@ -24641,7 +24675,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>264</v>
       </c>
@@ -24650,7 +24684,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>265</v>
       </c>
@@ -24659,12 +24693,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>268</v>
       </c>
@@ -24673,7 +24707,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>269</v>
       </c>
@@ -24682,7 +24716,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>270</v>
       </c>
@@ -24691,7 +24725,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13">
       <c r="D17" t="s">
         <v>275</v>
       </c>
@@ -24711,7 +24745,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13">
       <c r="A18" t="s">
         <v>551</v>
       </c>
@@ -24743,7 +24777,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13">
       <c r="A19" t="s">
         <v>552</v>
       </c>
@@ -24775,7 +24809,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13">
       <c r="A25" t="s">
         <v>278</v>
       </c>
@@ -24792,7 +24826,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13">
       <c r="A26" t="s">
         <v>263</v>
       </c>
@@ -24813,7 +24847,7 @@
         <v>472500</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13">
       <c r="A27" t="s">
         <v>264</v>
       </c>
@@ -24834,7 +24868,7 @@
         <v>680400</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13">
       <c r="A28" t="s">
         <v>265</v>
       </c>
@@ -24855,7 +24889,7 @@
         <v>267300</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5">
       <c r="A33" t="s">
         <v>286</v>
       </c>
@@ -24872,7 +24906,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5">
       <c r="A34" t="s">
         <v>275</v>
       </c>
@@ -24893,7 +24927,7 @@
         <v>2033100</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5">
       <c r="A35" t="s">
         <v>276</v>
       </c>
@@ -24914,7 +24948,7 @@
         <v>1703700</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
         <v>277</v>
       </c>
@@ -24935,7 +24969,7 @@
         <v>2284200</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5">
       <c r="A37" t="s">
         <v>283</v>
       </c>
@@ -24946,7 +24980,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{05C60535-1F16-4fd2-B633-F4F36F0B64E0}">
       <x14:sparklineGroups xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-        <x14:sparklineGroup displayEmptyCellsAs="gap">
+        <x14:sparklineGroup displayEmptyCellsAs="gap" xr2:uid="{00000000-0003-0000-0300-000001000000}">
           <x14:colorSeries rgb="FF376092"/>
           <x14:colorNegative rgb="FFD00000"/>
           <x14:colorAxis rgb="FF000000"/>

</xml_diff>